<commit_message>
update global estimate with temps
</commit_message>
<xml_diff>
--- a/data/ACSP_Data.xlsx
+++ b/data/ACSP_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27307"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27421"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://niva365.sharepoint.com/sites/int_AquaSYNC-SWG002-StefanoLarsenchair/Shared Documents/SWG002 - Stefano Larsen (chair)/Data/ACSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39E59017-2C59-421C-A179-29618ABD6E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3715E9F7-598F-45F2-9E25-0243CD4DA6BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9600" windowHeight="10200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9600" yWindow="0" windowWidth="9600" windowHeight="10200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="284">
   <si>
     <t>Index</t>
   </si>
@@ -226,9 +226,15 @@
     <t>Voshell_1985_NewRiver</t>
   </si>
   <si>
+    <t>Not able to find report</t>
+  </si>
+  <si>
     <t>Cross_EtAl_2006_C53_Reference</t>
   </si>
   <si>
+    <t>Nutrient addition. Include or not? (JSW: Yes...b/c we're interested in the range of production overall (and its variance), so this adds an estimate from a site with extra nutrients.)</t>
+  </si>
+  <si>
     <t>Cross_EtAl_2006_C54_NP_Enriched</t>
   </si>
   <si>
@@ -866,6 +872,18 @@
   </si>
   <si>
     <t>Shieh_EtAl_2002_CacheLaPoudreRiver_Site3</t>
+  </si>
+  <si>
+    <t>Benke_EtAl_1984_SatillaRiver_Lower</t>
+  </si>
+  <si>
+    <t>Applied habitat proportions from the text for snag:sand:mud habitat from pp50. Data are also available for Odonata, Coleoptera, and Oligochaeta. Width data probably an underestimate; likely excludes backwater "mud" habitat. Says basin size "more than double[s]" from upper to lower site.</t>
+  </si>
+  <si>
+    <t>Tables 4, 5, 6, 7, 8, 9, 10, 12, 13, 14, 15</t>
+  </si>
+  <si>
+    <t>Benke_EtAl_1984_SatillaRiver_Upper</t>
   </si>
   <si>
     <t>Index = copy from DataFileS1</t>
@@ -957,12 +975,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="8">
@@ -1080,7 +1116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1115,7 +1151,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1430,7 +1474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P172"/>
+  <dimension ref="A1:P174"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="48.42578125" bestFit="1" customWidth="1"/>
@@ -1815,7 +1859,7 @@
       <c r="E12">
         <v>2061</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="22">
         <f>SUM(G12:K12)</f>
         <v>1666.2</v>
       </c>
@@ -2179,54 +2223,61 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15" customHeight="1">
-      <c r="A23" s="2">
+    <row r="23" spans="1:14" s="20" customFormat="1" ht="15" customHeight="1">
+      <c r="A23" s="18">
         <v>143</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="19">
         <v>-80.885999999999996</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="19">
         <v>37.646000000000001</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" ht="15" customHeight="1">
-      <c r="A24" s="2">
+      <c r="M23" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" s="16" customFormat="1" ht="15" customHeight="1">
+      <c r="A24" s="14">
         <v>18</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="14">
+      <c r="B24" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="15">
         <v>-83.45</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="15">
         <v>35.06</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="2">
+      <c r="M24" s="17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" s="16" customFormat="1" ht="15" customHeight="1">
+      <c r="A25" s="14">
         <v>19</v>
       </c>
-      <c r="B25" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="14">
+      <c r="B25" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="15">
         <v>-83.44</v>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="15">
         <v>35.06</v>
       </c>
+      <c r="M25" s="17"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
       <c r="A26" s="2">
         <v>192</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C26" s="2">
         <v>170.32</v>
@@ -2257,7 +2308,7 @@
         <v>17</v>
       </c>
       <c r="M26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="15" customHeight="1">
@@ -2265,7 +2316,7 @@
         <v>105</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C27" s="2">
         <v>-96.57</v>
@@ -2301,7 +2352,7 @@
         <v>106</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C28" s="2">
         <v>-96.57</v>
@@ -2337,7 +2388,7 @@
         <v>107</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C29" s="2">
         <v>-96.57</v>
@@ -2373,7 +2424,7 @@
         <v>108</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C30" s="2">
         <v>-96.58</v>
@@ -2409,7 +2460,7 @@
         <v>109</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C31" s="2">
         <v>-96.58</v>
@@ -2445,7 +2496,7 @@
         <v>110</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C32" s="2">
         <v>-96.58</v>
@@ -2481,7 +2532,7 @@
         <v>46</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C33" s="2">
         <v>-83.4</v>
@@ -2493,50 +2544,50 @@
         <v>6</v>
       </c>
       <c r="L33" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M33" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="P33" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="15" customHeight="1">
       <c r="A34" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C34" s="2">
-        <v>-83.4</v>
+        <v>-83.46</v>
       </c>
       <c r="D34" s="2">
-        <v>35.06</v>
+        <v>35.04</v>
       </c>
       <c r="E34">
         <v>6</v>
       </c>
       <c r="L34" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M34" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="15" customHeight="1">
       <c r="A35" s="2">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C35" s="2">
         <v>-83.4</v>
       </c>
       <c r="D35" s="2">
-        <v>35.06</v>
+        <v>35.049999999999997</v>
       </c>
       <c r="E35">
         <v>5</v>
@@ -2546,24 +2597,24 @@
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
       <c r="L35" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M35" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:16" ht="15" customHeight="1">
       <c r="A36" s="2">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C36" s="2">
-        <v>-83.4</v>
+        <v>-83.45</v>
       </c>
       <c r="D36" s="2">
-        <v>35.06</v>
+        <v>35.04</v>
       </c>
       <c r="E36">
         <v>8</v>
@@ -2573,18 +2624,18 @@
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
       <c r="L36" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M36" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="15" customHeight="1">
       <c r="A37" s="2">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C37" s="2">
         <v>-83.4</v>
@@ -2600,21 +2651,21 @@
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
       <c r="L37" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M37" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="15" customHeight="1">
       <c r="A38" s="2">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C38" s="2">
-        <v>-83.4</v>
+        <v>-83.42</v>
       </c>
       <c r="D38" s="2">
         <v>35.06</v>
@@ -2627,24 +2678,24 @@
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
       <c r="L38" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M38" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="39" spans="1:16" ht="15" customHeight="1">
       <c r="A39" s="2">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C39" s="2">
-        <v>-83.4</v>
+        <v>-83.39</v>
       </c>
       <c r="D39" s="2">
-        <v>35.06</v>
+        <v>35.07</v>
       </c>
       <c r="E39">
         <v>21</v>
@@ -2654,24 +2705,24 @@
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
       <c r="L39" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M39" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="40" spans="1:16" ht="15" customHeight="1">
       <c r="A40" s="2">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C40" s="2">
-        <v>-83.4</v>
+        <v>-83.38</v>
       </c>
       <c r="D40" s="2">
-        <v>35.06</v>
+        <v>35.08</v>
       </c>
       <c r="E40">
         <v>7</v>
@@ -2681,24 +2732,24 @@
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
       <c r="L40" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M40" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="15" customHeight="1">
       <c r="A41" s="2">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C41" s="2">
-        <v>-83.4</v>
+        <v>-83.38</v>
       </c>
       <c r="D41" s="2">
-        <v>35.06</v>
+        <v>35.090000000000003</v>
       </c>
       <c r="E41">
         <v>22</v>
@@ -2708,24 +2759,24 @@
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
       <c r="L41" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M41" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="15" customHeight="1">
       <c r="A42" s="2">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C42" s="2">
-        <v>-83.4</v>
+        <v>-83.39</v>
       </c>
       <c r="D42" s="2">
-        <v>35.06</v>
+        <v>35.229999999999997</v>
       </c>
       <c r="E42">
         <v>154</v>
@@ -2735,24 +2786,24 @@
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
       <c r="L42" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M42" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:16" ht="15" customHeight="1">
       <c r="A43" s="2">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C43" s="2">
-        <v>-83.4</v>
+        <v>-83.52</v>
       </c>
       <c r="D43" s="2">
-        <v>35.06</v>
+        <v>35.33</v>
       </c>
       <c r="E43">
         <v>121</v>
@@ -2762,10 +2813,10 @@
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
       <c r="L43" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M43" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="15" customHeight="1">
@@ -2773,7 +2824,7 @@
         <v>197</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C44" s="2">
         <v>9.3330000000000002</v>
@@ -2803,13 +2854,13 @@
         <v>1.4</v>
       </c>
       <c r="L44" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="P44" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="15" customHeight="1">
@@ -2817,7 +2868,7 @@
         <v>155</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C45" s="2">
         <v>0.05</v>
@@ -2847,11 +2898,11 @@
         <v>0.51200000000000001</v>
       </c>
       <c r="L45" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M45" s="2"/>
       <c r="P45" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="46" spans="1:16" ht="15" customHeight="1">
@@ -2859,7 +2910,7 @@
         <v>111</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C46" s="2">
         <v>-85.98</v>
@@ -2875,13 +2926,13 @@
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
       <c r="L46" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="P46" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:16" ht="15" customHeight="1">
@@ -2889,7 +2940,7 @@
         <v>112</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C47" s="2">
         <v>-85.98</v>
@@ -2905,13 +2956,13 @@
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
       <c r="L47" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="P47" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="48" spans="1:16" ht="15" customHeight="1">
@@ -2919,7 +2970,7 @@
         <v>113</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C48" s="2">
         <v>-85.98</v>
@@ -2935,13 +2986,13 @@
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="L48" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="P48" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="49" spans="1:16" ht="15" customHeight="1">
@@ -2949,7 +3000,7 @@
         <v>79</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C49" s="2">
         <v>-105.63</v>
@@ -2980,12 +3031,12 @@
         <v>20</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:16" ht="15" customHeight="1">
@@ -2993,7 +3044,7 @@
         <v>79</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C50" s="2">
         <v>-105.63</v>
@@ -3024,12 +3075,12 @@
         <v>20</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="51" spans="1:16" ht="15" customHeight="1">
@@ -3037,7 +3088,7 @@
         <v>80</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C51" s="2">
         <v>-105.44</v>
@@ -3068,10 +3119,10 @@
         <v>20</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="P51" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="52" spans="1:16" ht="15" customHeight="1">
@@ -3079,7 +3130,7 @@
         <v>80</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C52" s="2">
         <v>-105.44</v>
@@ -3110,10 +3161,10 @@
         <v>20</v>
       </c>
       <c r="M52" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="P52" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="P52" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="53" spans="1:16" ht="15" customHeight="1">
@@ -3121,7 +3172,7 @@
         <v>81</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C53" s="2">
         <v>-105.52</v>
@@ -3152,10 +3203,10 @@
         <v>20</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="P53" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="15" customHeight="1">
@@ -3163,7 +3214,7 @@
         <v>81</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C54" s="2">
         <v>-105.52</v>
@@ -3194,10 +3245,10 @@
         <v>20</v>
       </c>
       <c r="M54" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="P54" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="P54" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:16" ht="15" customHeight="1">
@@ -3205,7 +3256,7 @@
         <v>82</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C55" s="2">
         <v>-105.63</v>
@@ -3236,10 +3287,10 @@
         <v>20</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="P55" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56" spans="1:16" ht="15" customHeight="1">
@@ -3247,7 +3298,7 @@
         <v>82</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C56" s="2">
         <v>-105.63</v>
@@ -3278,10 +3329,10 @@
         <v>20</v>
       </c>
       <c r="M56" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="P56" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="P56" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="57" spans="1:16" ht="15" customHeight="1">
@@ -3289,7 +3340,7 @@
         <v>28</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C57" s="2">
         <v>-88.9</v>
@@ -3301,16 +3352,16 @@
         <v>0.9</v>
       </c>
       <c r="L57" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="N57">
         <v>2.4</v>
       </c>
       <c r="P57" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:16" ht="15" customHeight="1">
@@ -3318,7 +3369,7 @@
         <v>28</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C58" s="2">
         <v>-88.9</v>
@@ -3330,13 +3381,13 @@
         <v>1.5</v>
       </c>
       <c r="L58" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N58">
         <v>2.5</v>
       </c>
       <c r="P58" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:16" ht="15" customHeight="1">
@@ -3344,7 +3395,7 @@
         <v>28</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C59" s="2">
         <v>-88.9</v>
@@ -3356,13 +3407,13 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="L59" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N59">
         <v>2.5</v>
       </c>
       <c r="P59" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60" spans="1:16" ht="15" customHeight="1">
@@ -3370,7 +3421,7 @@
         <v>30</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C60" s="2">
         <v>-88.9</v>
@@ -3382,16 +3433,16 @@
         <v>3.1</v>
       </c>
       <c r="L60" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="N60">
         <v>2.1</v>
       </c>
       <c r="P60" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61" spans="1:16" ht="15" customHeight="1">
@@ -3399,7 +3450,7 @@
         <v>30</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C61" s="2">
         <v>-88.9</v>
@@ -3411,13 +3462,13 @@
         <v>1.6</v>
       </c>
       <c r="L61" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N61">
         <v>2.2999999999999998</v>
       </c>
       <c r="P61" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="62" spans="1:16" ht="15" customHeight="1">
@@ -3425,7 +3476,7 @@
         <v>30</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C62" s="2">
         <v>-88.9</v>
@@ -3437,13 +3488,13 @@
         <v>2.7</v>
       </c>
       <c r="L62" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N62">
         <v>2.2999999999999998</v>
       </c>
       <c r="P62" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="63" spans="1:16" ht="15" customHeight="1">
@@ -3451,7 +3502,7 @@
         <v>32</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C63" s="2">
         <v>-88.9</v>
@@ -3463,16 +3514,16 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="L63" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="N63">
         <v>1.8</v>
       </c>
       <c r="P63" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64" spans="1:16" ht="15" customHeight="1">
@@ -3480,7 +3531,7 @@
         <v>32</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C64" s="2">
         <v>-88.9</v>
@@ -3492,13 +3543,13 @@
         <v>1.3</v>
       </c>
       <c r="L64" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N64">
         <v>2.4</v>
       </c>
       <c r="P64" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65" spans="1:16" ht="15" customHeight="1">
@@ -3506,7 +3557,7 @@
         <v>32</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C65" s="2">
         <v>-88.9</v>
@@ -3518,13 +3569,13 @@
         <v>0.9</v>
       </c>
       <c r="L65" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N65">
         <v>2.4</v>
       </c>
       <c r="P65" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="66" spans="1:16" ht="15" customHeight="1">
@@ -3532,7 +3583,7 @@
         <v>9</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C66" s="2">
         <v>-68.13</v>
@@ -3562,7 +3613,7 @@
         <v>17</v>
       </c>
       <c r="P66" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:16" ht="15" customHeight="1">
@@ -3570,7 +3621,7 @@
         <v>10</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C67" s="2">
         <v>-68.13</v>
@@ -3600,7 +3651,7 @@
         <v>17</v>
       </c>
       <c r="P67" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="68" spans="1:16" ht="15" customHeight="1">
@@ -3608,7 +3659,7 @@
         <v>11</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C68" s="2">
         <v>-68.14</v>
@@ -3638,7 +3689,7 @@
         <v>17</v>
       </c>
       <c r="P68" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="69" spans="1:16" ht="15" customHeight="1">
@@ -3646,7 +3697,7 @@
         <v>12</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C69" s="2">
         <v>-68.14</v>
@@ -3676,7 +3727,7 @@
         <v>17</v>
       </c>
       <c r="P69" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="70" spans="1:16" ht="15" customHeight="1">
@@ -3684,7 +3735,7 @@
         <v>131</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C70" s="2">
         <v>-68.12</v>
@@ -3696,13 +3747,13 @@
         <v>1.68</v>
       </c>
       <c r="L70" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M70" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P70" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" spans="1:16" ht="15" customHeight="1">
@@ -3710,7 +3761,7 @@
         <v>13</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C71" s="2">
         <v>-68.12</v>
@@ -3722,13 +3773,13 @@
         <v>2</v>
       </c>
       <c r="L71" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M71" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P71" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" spans="1:16" ht="15" customHeight="1">
@@ -3736,7 +3787,7 @@
         <v>14</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C72" s="2">
         <v>-68.12</v>
@@ -3748,13 +3799,13 @@
         <v>2.19</v>
       </c>
       <c r="L72" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M72" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P72" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="73" spans="1:16" ht="15" customHeight="1">
@@ -3762,7 +3813,7 @@
         <v>15</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C73" s="2">
         <v>-68.099999999999994</v>
@@ -3774,13 +3825,13 @@
         <v>2.89</v>
       </c>
       <c r="L73" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M73" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P73" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" spans="1:16" ht="15" customHeight="1">
@@ -3788,7 +3839,7 @@
         <v>16</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C74" s="2">
         <v>-68.12</v>
@@ -3800,13 +3851,13 @@
         <v>2.09</v>
       </c>
       <c r="L74" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M74" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P74" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="75" spans="1:16" ht="15" customHeight="1">
@@ -3814,7 +3865,7 @@
         <v>17</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C75" s="2">
         <v>-68.14</v>
@@ -3826,13 +3877,13 @@
         <v>1.65</v>
       </c>
       <c r="L75" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M75" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P75" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="76" spans="1:16" ht="15" customHeight="1">
@@ -3840,7 +3891,7 @@
         <v>41</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C76" s="2">
         <v>-83.43</v>
@@ -3850,7 +3901,7 @@
       </c>
       <c r="L76" s="12"/>
       <c r="M76" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="N76">
         <v>5.5</v>
@@ -3861,7 +3912,7 @@
         <v>75</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C77" s="2">
         <v>-112.25</v>
@@ -3894,13 +3945,13 @@
         <v>17</v>
       </c>
       <c r="M77" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="N77">
         <v>3.5</v>
       </c>
       <c r="P77" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="78" spans="1:16" ht="15" customHeight="1">
@@ -3908,7 +3959,7 @@
         <v>35</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C78" s="2">
         <v>-111.5</v>
@@ -3917,7 +3968,7 @@
         <v>33.75</v>
       </c>
       <c r="M78" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="79" spans="1:16" ht="15" customHeight="1">
@@ -3925,7 +3976,7 @@
         <v>186</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C79" s="2">
         <v>174.9</v>
@@ -3943,10 +3994,10 @@
       <c r="J79" s="5"/>
       <c r="K79" s="5"/>
       <c r="L79" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M79" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N79" s="6"/>
     </row>
@@ -3955,7 +4006,7 @@
         <v>187</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C80" s="2">
         <v>174.9</v>
@@ -3973,10 +4024,10 @@
       <c r="J80" s="5"/>
       <c r="K80" s="5"/>
       <c r="L80" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M80" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N80" s="6"/>
     </row>
@@ -3985,7 +4036,7 @@
         <v>188</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C81" s="2">
         <v>174.9</v>
@@ -4003,10 +4054,10 @@
       <c r="J81" s="5"/>
       <c r="K81" s="5"/>
       <c r="L81" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M81" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N81" s="6"/>
     </row>
@@ -4015,7 +4066,7 @@
         <v>189</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C82" s="2">
         <v>175.483</v>
@@ -4033,10 +4084,10 @@
       <c r="J82" s="5"/>
       <c r="K82" s="5"/>
       <c r="L82" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M82" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N82" s="6"/>
     </row>
@@ -4045,7 +4096,7 @@
         <v>190</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C83" s="2">
         <v>175.483</v>
@@ -4063,10 +4114,10 @@
       <c r="J83" s="5"/>
       <c r="K83" s="5"/>
       <c r="L83" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M83" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N83" s="6"/>
     </row>
@@ -4075,7 +4126,7 @@
         <v>191</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C84" s="2">
         <v>175.483</v>
@@ -4093,10 +4144,10 @@
       <c r="J84" s="5"/>
       <c r="K84" s="5"/>
       <c r="L84" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M84" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N84" s="6"/>
     </row>
@@ -4105,7 +4156,7 @@
         <v>61</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C85" s="2">
         <v>-81.099999999999994</v>
@@ -4131,10 +4182,10 @@
       </c>
       <c r="K85" s="5"/>
       <c r="L85" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M85" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N85" s="6"/>
     </row>
@@ -4143,7 +4194,7 @@
         <v>62</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C86" s="2">
         <v>-81.19</v>
@@ -4167,10 +4218,10 @@
       </c>
       <c r="K86" s="5"/>
       <c r="L86" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M86" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N86" s="6"/>
     </row>
@@ -4179,7 +4230,7 @@
         <v>65</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C87" s="2">
         <v>-81.040000000000006</v>
@@ -4203,10 +4254,10 @@
       </c>
       <c r="K87" s="5"/>
       <c r="L87" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M87" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N87" s="6"/>
     </row>
@@ -4215,7 +4266,7 @@
         <v>67</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C88" s="2">
         <v>-81.12</v>
@@ -4241,10 +4292,10 @@
       </c>
       <c r="K88" s="5"/>
       <c r="L88" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M88" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N88" s="6"/>
     </row>
@@ -4253,7 +4304,7 @@
         <v>68</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C89" s="2">
         <v>-81.11</v>
@@ -4279,10 +4330,10 @@
       </c>
       <c r="K89" s="5"/>
       <c r="L89" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M89" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N89" s="6"/>
     </row>
@@ -4291,7 +4342,7 @@
         <v>70</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C90" s="2">
         <v>-81.08</v>
@@ -4317,10 +4368,10 @@
       </c>
       <c r="K90" s="5"/>
       <c r="L90" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N90" s="6"/>
     </row>
@@ -4329,7 +4380,7 @@
         <v>71</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C91" s="2">
         <v>-81.040000000000006</v>
@@ -4355,10 +4406,10 @@
       </c>
       <c r="K91" s="5"/>
       <c r="L91" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M91" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N91" s="6"/>
     </row>
@@ -4367,7 +4418,7 @@
         <v>73</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C92" s="2">
         <v>-81.03</v>
@@ -4391,10 +4442,10 @@
         <v>6.3</v>
       </c>
       <c r="L92" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M92" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N92" s="6"/>
     </row>
@@ -4403,7 +4454,7 @@
         <v>136</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C93" s="2">
         <v>-81.049000000000007</v>
@@ -4427,10 +4478,10 @@
       </c>
       <c r="K93" s="5"/>
       <c r="L93" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M93" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N93" s="6"/>
     </row>
@@ -4439,7 +4490,7 @@
         <v>137</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C94" s="2">
         <v>-81.037999999999997</v>
@@ -4463,10 +4514,10 @@
       </c>
       <c r="K94" s="5"/>
       <c r="L94" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M94" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N94" s="6"/>
     </row>
@@ -4475,7 +4526,7 @@
         <v>144</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C95" s="2">
         <v>-110.83499999999999</v>
@@ -4515,7 +4566,7 @@
         <v>145</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C96" s="2">
         <v>-110.836</v>
@@ -4555,7 +4606,7 @@
         <v>146</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C97" s="2">
         <v>-110.687</v>
@@ -4595,7 +4646,7 @@
         <v>147</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C98" s="2">
         <v>-110.855</v>
@@ -4635,7 +4686,7 @@
         <v>21</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C99" s="2">
         <v>-111.85</v>
@@ -4665,10 +4716,10 @@
         <v>5.7781000000000002</v>
       </c>
       <c r="L99" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M99" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N99" s="6"/>
     </row>
@@ -4677,7 +4728,7 @@
         <v>22</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C100" s="2">
         <v>-111.81</v>
@@ -4707,10 +4758,10 @@
         <v>0.28206666670000002</v>
       </c>
       <c r="L100" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M100" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N100" s="6"/>
     </row>
@@ -4719,7 +4770,7 @@
         <v>23</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C101" s="2">
         <v>-112.49</v>
@@ -4749,10 +4800,10 @@
         <v>0.52370000000000005</v>
       </c>
       <c r="L101" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M101" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N101" s="6"/>
     </row>
@@ -4761,7 +4812,7 @@
         <v>24</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C102" s="2">
         <v>-112.85</v>
@@ -4791,10 +4842,10 @@
         <v>0.57506666669999995</v>
       </c>
       <c r="L102" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M102" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N102" s="6"/>
     </row>
@@ -4803,7 +4854,7 @@
         <v>25</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C103" s="2">
         <v>-113.36</v>
@@ -4833,10 +4884,10 @@
         <v>0.53563333329999996</v>
       </c>
       <c r="L103" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M103" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N103" s="6"/>
     </row>
@@ -4845,7 +4896,7 @@
         <v>4</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C104" s="2">
         <v>-105.86</v>
@@ -4885,7 +4936,7 @@
         <v>5</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C105" s="2">
         <v>-106.07</v>
@@ -4925,7 +4976,7 @@
         <v>6</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C106" s="2">
         <v>-106.07</v>
@@ -4965,7 +5016,7 @@
         <v>7</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C107" s="2">
         <v>-106.21</v>
@@ -5005,7 +5056,7 @@
         <v>8</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C108" s="2">
         <v>-106.08</v>
@@ -5045,7 +5096,7 @@
         <v>114</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C109" s="2">
         <v>-83.45</v>
@@ -5066,7 +5117,7 @@
         <v>17</v>
       </c>
       <c r="M109" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="N109" s="6"/>
     </row>
@@ -5075,7 +5126,7 @@
         <v>115</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C110" s="2">
         <v>-83.45</v>
@@ -5096,7 +5147,7 @@
         <v>17</v>
       </c>
       <c r="M110" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="N110" s="6"/>
     </row>
@@ -5105,7 +5156,7 @@
         <v>116</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C111" s="2">
         <v>-83.45</v>
@@ -5126,7 +5177,7 @@
         <v>17</v>
       </c>
       <c r="M111" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="N111" s="6"/>
     </row>
@@ -5135,7 +5186,7 @@
         <v>117</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C112" s="2">
         <v>-83.45</v>
@@ -5156,7 +5207,7 @@
         <v>17</v>
       </c>
       <c r="M112" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="N112" s="10"/>
     </row>
@@ -5165,7 +5216,7 @@
         <v>149</v>
       </c>
       <c r="B113" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C113" s="2">
         <v>-91.037000000000006</v>
@@ -5189,10 +5240,10 @@
         <v>4.24</v>
       </c>
       <c r="L113" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="M113" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="N113">
         <v>4.5</v>
@@ -5203,7 +5254,7 @@
         <v>150</v>
       </c>
       <c r="B114" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C114" s="2">
         <v>-92.561000000000007</v>
@@ -5227,10 +5278,10 @@
         <v>37.472000000000001</v>
       </c>
       <c r="L114" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="M114" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="N114">
         <v>6</v>
@@ -5241,7 +5292,7 @@
         <v>151</v>
       </c>
       <c r="B115" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C115" s="2">
         <v>-92.531000000000006</v>
@@ -5265,10 +5316,10 @@
         <v>15.851000000000001</v>
       </c>
       <c r="L115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="M115" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="N115">
         <v>5.5</v>
@@ -5279,7 +5330,7 @@
         <v>167</v>
       </c>
       <c r="B116" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C116" s="2">
         <v>-80.582999999999998</v>
@@ -5306,13 +5357,13 @@
         <v>17</v>
       </c>
       <c r="M116" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="N116">
         <v>3.28</v>
       </c>
       <c r="P116" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="117" spans="1:16" ht="15" customHeight="1">
@@ -5320,7 +5371,7 @@
         <v>168</v>
       </c>
       <c r="B117" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C117" s="2">
         <v>-80.582999999999998</v>
@@ -5350,7 +5401,7 @@
         <v>3.55</v>
       </c>
       <c r="P117" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="118" spans="1:16" ht="15" customHeight="1">
@@ -5358,7 +5409,7 @@
         <v>169</v>
       </c>
       <c r="B118" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C118" s="2">
         <v>-80.233000000000004</v>
@@ -5388,7 +5439,7 @@
         <v>3.37</v>
       </c>
       <c r="P118" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="119" spans="1:16" ht="15" customHeight="1">
@@ -5396,7 +5447,7 @@
         <v>170</v>
       </c>
       <c r="B119" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C119" s="2">
         <v>-80.233000000000004</v>
@@ -5426,7 +5477,7 @@
         <v>2.0099999999999998</v>
       </c>
       <c r="P119" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="120" spans="1:16" ht="15" customHeight="1">
@@ -5434,7 +5485,7 @@
         <v>78</v>
       </c>
       <c r="B120" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C120" s="2">
         <v>-118.83</v>
@@ -5461,10 +5512,10 @@
         <v>0.12</v>
       </c>
       <c r="L120" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P120" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="121" spans="1:16" ht="15" customHeight="1">
@@ -5472,7 +5523,7 @@
         <v>83</v>
       </c>
       <c r="B121" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C121" s="2">
         <v>-79.510000000000005</v>
@@ -5496,16 +5547,16 @@
         <v>0.05</v>
       </c>
       <c r="L121" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M121" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N121">
         <v>3</v>
       </c>
       <c r="P121" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="122" spans="1:16" ht="15" customHeight="1">
@@ -5513,7 +5564,7 @@
         <v>84</v>
       </c>
       <c r="B122" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C122" s="2">
         <v>-79.5</v>
@@ -5537,16 +5588,16 @@
         <v>9.74</v>
       </c>
       <c r="L122" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M122" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N122">
         <v>5.3</v>
       </c>
       <c r="P122" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="123" spans="1:16" ht="15" customHeight="1">
@@ -5554,7 +5605,7 @@
         <v>85</v>
       </c>
       <c r="B123" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C123" s="2">
         <v>-79.48</v>
@@ -5578,16 +5629,16 @@
         <v>6.62</v>
       </c>
       <c r="L123" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M123" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N123">
         <v>6.1</v>
       </c>
       <c r="P123" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="124" spans="1:16" ht="15" customHeight="1">
@@ -5595,7 +5646,7 @@
         <v>86</v>
       </c>
       <c r="B124" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C124" s="2">
         <v>-79.47</v>
@@ -5619,16 +5670,16 @@
         <v>2.2400000000000002</v>
       </c>
       <c r="L124" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M124" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N124">
         <v>5.6</v>
       </c>
       <c r="P124" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="125" spans="1:16" ht="15" customHeight="1">
@@ -5636,7 +5687,7 @@
         <v>87</v>
       </c>
       <c r="B125" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C125" s="2">
         <v>-79.489999999999995</v>
@@ -5660,16 +5711,16 @@
         <v>0</v>
       </c>
       <c r="L125" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M125" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N125">
         <v>2.9</v>
       </c>
       <c r="P125" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="126" spans="1:16" ht="15" customHeight="1">
@@ -5677,7 +5728,7 @@
         <v>158</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C126" s="2">
         <v>-67.655000000000001</v>
@@ -5697,7 +5748,7 @@
         <v>159</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C127" s="2">
         <v>-67.655000000000001</v>
@@ -5712,7 +5763,7 @@
         <v>17</v>
       </c>
       <c r="M127" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="128" spans="1:16" ht="15" customHeight="1">
@@ -5720,7 +5771,7 @@
         <v>160</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C128" s="2">
         <v>-67.655000000000001</v>
@@ -5735,7 +5786,7 @@
         <v>17</v>
       </c>
       <c r="M128" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="129" spans="1:16" ht="15" customHeight="1">
@@ -5743,7 +5794,7 @@
         <v>138</v>
       </c>
       <c r="B129" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C129" s="2">
         <v>-83.46</v>
@@ -5767,10 +5818,10 @@
         <v>2.93</v>
       </c>
       <c r="L129" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M129" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="130" spans="1:16" ht="15" customHeight="1">
@@ -5778,7 +5829,7 @@
         <v>139</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C130" s="2">
         <v>-83.465999999999994</v>
@@ -5802,10 +5853,10 @@
         <v>1.85</v>
       </c>
       <c r="L130" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M130" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="131" spans="1:16" ht="15" customHeight="1">
@@ -5813,7 +5864,7 @@
         <v>140</v>
       </c>
       <c r="B131" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C131" s="2">
         <v>-83.465999999999994</v>
@@ -5831,10 +5882,10 @@
         <v>0.08</v>
       </c>
       <c r="L131" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M131" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="132" spans="1:16" ht="15" customHeight="1">
@@ -5842,7 +5893,7 @@
         <v>141</v>
       </c>
       <c r="B132" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C132" s="2">
         <v>-83.456999999999994</v>
@@ -5866,10 +5917,10 @@
         <v>1.59</v>
       </c>
       <c r="L132" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M132" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="133" spans="1:16" ht="15" customHeight="1">
@@ -5877,7 +5928,7 @@
         <v>142</v>
       </c>
       <c r="B133" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C133" s="2">
         <v>-83.456999999999994</v>
@@ -5901,10 +5952,10 @@
         <v>1.71</v>
       </c>
       <c r="L133" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M133" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="134" spans="1:16" ht="15" customHeight="1">
@@ -5912,7 +5963,7 @@
         <v>97</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C134" s="2">
         <v>-105</v>
@@ -5930,15 +5981,15 @@
       <c r="J134" s="2"/>
       <c r="K134" s="2"/>
       <c r="L134" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M134" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="N134" s="2"/>
       <c r="O134" s="2"/>
       <c r="P134" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="135" spans="1:16" ht="15" customHeight="1">
@@ -5946,7 +5997,7 @@
         <v>98</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C135" s="2">
         <v>-104.99</v>
@@ -5964,15 +6015,15 @@
       <c r="J135" s="2"/>
       <c r="K135" s="2"/>
       <c r="L135" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M135" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="N135" s="2"/>
       <c r="O135" s="2"/>
       <c r="P135" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="136" spans="1:16" ht="15" customHeight="1">
@@ -5980,7 +6031,7 @@
         <v>99</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C136" s="2">
         <v>-104.98</v>
@@ -5998,15 +6049,15 @@
       <c r="J136" s="2"/>
       <c r="K136" s="2"/>
       <c r="L136" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M136" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="N136" s="2"/>
       <c r="O136" s="2"/>
       <c r="P136" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="137" spans="1:16" ht="15" customHeight="1">
@@ -6014,7 +6065,7 @@
         <v>26</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C137" s="2">
         <v>-83.43</v>
@@ -6035,14 +6086,14 @@
         <v>17</v>
       </c>
       <c r="M137" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N137" s="2"/>
       <c r="O137" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="P137" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="138" spans="1:16" ht="15" customHeight="1">
@@ -6050,7 +6101,7 @@
         <v>27</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C138" s="2">
         <v>-83.43</v>
@@ -6071,14 +6122,14 @@
         <v>17</v>
       </c>
       <c r="M138" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N138" s="2"/>
       <c r="O138" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="P138" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="P138" s="2" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="139" spans="1:16" ht="15" customHeight="1">
@@ -6086,7 +6137,7 @@
         <v>103</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C139" s="2">
         <v>-83.43</v>
@@ -6107,14 +6158,14 @@
         <v>17</v>
       </c>
       <c r="M139" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="N139" s="2"/>
       <c r="O139" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="P139" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="140" spans="1:16" ht="15" customHeight="1">
@@ -6122,7 +6173,7 @@
         <v>104</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C140" s="2">
         <v>-83.43</v>
@@ -6143,14 +6194,14 @@
         <v>17</v>
       </c>
       <c r="M140" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="N140" s="2"/>
       <c r="O140" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="P140" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="P140" s="2" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="141" spans="1:16" ht="14.45">
@@ -6158,7 +6209,7 @@
         <v>100</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C141" s="2">
         <v>-77.09</v>
@@ -6170,16 +6221,16 @@
         <v>5.6</v>
       </c>
       <c r="L141" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M141" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="N141">
         <v>2.5</v>
       </c>
       <c r="P141" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="142" spans="1:16" ht="14.45">
@@ -6187,7 +6238,7 @@
         <v>101</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C142" s="2">
         <v>-77.03</v>
@@ -6199,16 +6250,16 @@
         <v>6.2</v>
       </c>
       <c r="L142" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M142" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="N142">
         <v>3</v>
       </c>
       <c r="P142" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="143" spans="1:16" ht="15" customHeight="1">
@@ -6216,7 +6267,7 @@
         <v>89</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C143" s="2">
         <v>-112.88</v>
@@ -6242,17 +6293,17 @@
         <v>5.44</v>
       </c>
       <c r="L143" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M143" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="N143" s="2">
         <v>10</v>
       </c>
       <c r="O143" s="2"/>
       <c r="P143" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="144" spans="1:16" ht="15" customHeight="1">
@@ -6260,7 +6311,7 @@
         <v>90</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C144" s="2">
         <v>-113.21</v>
@@ -6286,17 +6337,17 @@
         <v>0.27</v>
       </c>
       <c r="L144" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M144" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="N144" s="2">
         <v>7.5</v>
       </c>
       <c r="O144" s="2"/>
       <c r="P144" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="145" spans="1:16" ht="15" customHeight="1">
@@ -6304,7 +6355,7 @@
         <v>66</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C145" s="2">
         <v>-85.62</v>
@@ -6325,7 +6376,7 @@
         <v>17</v>
       </c>
       <c r="M145" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="N145" s="2">
         <v>4.5</v>
@@ -6334,7 +6385,7 @@
         <v>7.3</v>
       </c>
       <c r="P145" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="146" spans="1:16" ht="15" customHeight="1">
@@ -6342,7 +6393,7 @@
         <v>74</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C146" s="2">
         <v>-85.75</v>
@@ -6363,7 +6414,7 @@
         <v>17</v>
       </c>
       <c r="M146" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="N146" s="2">
         <v>4.8</v>
@@ -6372,7 +6423,7 @@
         <v>14.8</v>
       </c>
       <c r="P146" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="147" spans="1:16" ht="15" customHeight="1">
@@ -6380,7 +6431,7 @@
         <v>72</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C147" s="2">
         <v>-86.29</v>
@@ -6401,7 +6452,7 @@
         <v>17</v>
       </c>
       <c r="M147" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="N147" s="2">
         <v>5.6</v>
@@ -6410,7 +6461,7 @@
         <v>5.3</v>
       </c>
       <c r="P147" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="148" spans="1:16" ht="15" customHeight="1">
@@ -6418,7 +6469,7 @@
         <v>69</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C148" s="2">
         <v>-85.61</v>
@@ -6439,7 +6490,7 @@
         <v>17</v>
       </c>
       <c r="M148" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="N148" s="2">
         <v>6.3</v>
@@ -6448,7 +6499,7 @@
         <v>15</v>
       </c>
       <c r="P148" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="149" spans="1:16" ht="15" customHeight="1">
@@ -6456,7 +6507,7 @@
         <v>64</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C149" s="2">
         <v>-85.56</v>
@@ -6477,7 +6528,7 @@
         <v>17</v>
       </c>
       <c r="M149" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="N149" s="2">
         <v>5.9</v>
@@ -6486,7 +6537,7 @@
         <v>3.1</v>
       </c>
       <c r="P149" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="150" spans="1:16" ht="15" customHeight="1">
@@ -6494,7 +6545,7 @@
         <v>63</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C150" s="2">
         <v>-85.56</v>
@@ -6515,7 +6566,7 @@
         <v>17</v>
       </c>
       <c r="M150" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="N150" s="2">
         <v>3.6</v>
@@ -6524,7 +6575,7 @@
         <v>4.3</v>
       </c>
       <c r="P150" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="151" spans="1:16" ht="15" customHeight="1">
@@ -6532,7 +6583,7 @@
         <v>102</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C151" s="2">
         <v>-96.58</v>
@@ -6563,16 +6614,16 @@
         <v>17</v>
       </c>
       <c r="M151" s="2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="N151" s="2">
         <v>1.6</v>
       </c>
       <c r="O151" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="P151" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="152" spans="1:16" ht="15" customHeight="1">
@@ -6580,7 +6631,7 @@
         <v>152</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C152" s="2">
         <v>-80.832999999999998</v>
@@ -6601,12 +6652,12 @@
         <v>20</v>
       </c>
       <c r="M152" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="N152" s="2"/>
       <c r="O152" s="2"/>
       <c r="P152" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="153" spans="1:16" ht="15" customHeight="1">
@@ -6614,7 +6665,7 @@
         <v>153</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C153" s="2">
         <v>-80.828999999999994</v>
@@ -6635,12 +6686,12 @@
         <v>20</v>
       </c>
       <c r="M153" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="N153" s="2"/>
       <c r="O153" s="2"/>
       <c r="P153" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="154" spans="1:16" ht="15" customHeight="1">
@@ -6648,7 +6699,7 @@
         <v>154</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C154" s="2">
         <v>-80.822999999999993</v>
@@ -6669,12 +6720,12 @@
         <v>20</v>
       </c>
       <c r="M154" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="N154" s="2"/>
       <c r="O154" s="2"/>
       <c r="P154" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="155" spans="1:16" ht="15" customHeight="1">
@@ -6682,7 +6733,7 @@
         <v>220</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C155" s="2">
         <v>-1.35</v>
@@ -6710,17 +6761,17 @@
       </c>
       <c r="K155" s="2"/>
       <c r="L155" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M155" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="N155" s="2">
         <v>4.5</v>
       </c>
       <c r="O155" s="2"/>
       <c r="P155" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="156" spans="1:16" ht="15" customHeight="1">
@@ -6728,7 +6779,7 @@
         <v>221</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C156" s="2">
         <v>-1.35</v>
@@ -6756,17 +6807,17 @@
       </c>
       <c r="K156" s="2"/>
       <c r="L156" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M156" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="N156" s="2">
         <v>4.5</v>
       </c>
       <c r="O156" s="2"/>
       <c r="P156" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="157" spans="1:16" ht="15" customHeight="1">
@@ -6774,7 +6825,7 @@
         <v>34</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C157" s="2">
         <v>-72.510000000000005</v>
@@ -6792,7 +6843,7 @@
       <c r="J157" s="2"/>
       <c r="K157" s="2"/>
       <c r="L157" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M157" s="2"/>
       <c r="N157" s="2">
@@ -6802,7 +6853,7 @@
         <v>105</v>
       </c>
       <c r="P157" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="158" spans="1:16" ht="15" customHeight="1">
@@ -6810,7 +6861,7 @@
         <v>129</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C158" s="2">
         <v>-96.58</v>
@@ -6831,7 +6882,7 @@
         <v>17</v>
       </c>
       <c r="M158" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="N158" s="2">
         <v>0.7</v>
@@ -6840,7 +6891,7 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="P158" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="159" spans="1:16" ht="15" customHeight="1">
@@ -6848,7 +6899,7 @@
         <v>130</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C159" s="2">
         <v>-96.58</v>
@@ -6869,7 +6920,7 @@
         <v>17</v>
       </c>
       <c r="M159" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="N159" s="2">
         <v>0.9</v>
@@ -6878,7 +6929,7 @@
         <v>1.34</v>
       </c>
       <c r="P159" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="160" spans="1:16" ht="15" customHeight="1">
@@ -6886,7 +6937,7 @@
         <v>128</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C160" s="2">
         <v>-96.61</v>
@@ -6907,7 +6958,7 @@
         <v>17</v>
       </c>
       <c r="M160" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="N160" s="2">
         <v>1.6</v>
@@ -6916,7 +6967,7 @@
         <v>10.59</v>
       </c>
       <c r="P160" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="161" spans="1:16" ht="14.45">
@@ -6924,7 +6975,7 @@
         <v>179</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C161">
         <v>-21.3</v>
@@ -6939,10 +6990,10 @@
         <v>20</v>
       </c>
       <c r="M161" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="P161" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="162" spans="1:16" ht="14.45">
@@ -6950,7 +7001,7 @@
         <v>180</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C162">
         <v>-21.3</v>
@@ -6965,10 +7016,10 @@
         <v>20</v>
       </c>
       <c r="M162" t="s">
+        <v>252</v>
+      </c>
+      <c r="P162" t="s">
         <v>250</v>
-      </c>
-      <c r="P162" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="163" spans="1:16" ht="14.45">
@@ -6976,7 +7027,7 @@
         <v>181</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C163">
         <v>-21.3</v>
@@ -6991,10 +7042,10 @@
         <v>20</v>
       </c>
       <c r="M163" t="s">
+        <v>252</v>
+      </c>
+      <c r="P163" t="s">
         <v>250</v>
-      </c>
-      <c r="P163" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="164" spans="1:16" ht="14.45">
@@ -7002,7 +7053,7 @@
         <v>182</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C164">
         <v>-21.3</v>
@@ -7017,10 +7068,10 @@
         <v>20</v>
       </c>
       <c r="M164" t="s">
+        <v>252</v>
+      </c>
+      <c r="P164" t="s">
         <v>250</v>
-      </c>
-      <c r="P164" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="165" spans="1:16" ht="14.45">
@@ -7028,7 +7079,7 @@
         <v>183</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C165">
         <v>-21.3</v>
@@ -7043,10 +7094,10 @@
         <v>20</v>
       </c>
       <c r="M165" t="s">
+        <v>252</v>
+      </c>
+      <c r="P165" t="s">
         <v>250</v>
-      </c>
-      <c r="P165" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="166" spans="1:16" ht="14.45">
@@ -7054,7 +7105,7 @@
         <v>184</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C166">
         <v>-21.3</v>
@@ -7069,10 +7120,10 @@
         <v>20</v>
       </c>
       <c r="M166" t="s">
+        <v>252</v>
+      </c>
+      <c r="P166" t="s">
         <v>250</v>
-      </c>
-      <c r="P166" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="167" spans="1:16" ht="14.45">
@@ -7080,7 +7131,7 @@
         <v>133</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C167">
         <v>-82.507999999999996</v>
@@ -7092,10 +7143,10 @@
         <v>7.4</v>
       </c>
       <c r="L167" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M167" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="N167">
         <v>250</v>
@@ -7104,7 +7155,7 @@
         <v>579000</v>
       </c>
       <c r="P167" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="168" spans="1:16" ht="14.45">
@@ -7112,7 +7163,7 @@
         <v>134</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C168">
         <v>-83.084000000000003</v>
@@ -7124,10 +7175,10 @@
         <v>5.4</v>
       </c>
       <c r="L168" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M168" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="N168">
         <v>3000</v>
@@ -7136,7 +7187,7 @@
         <v>598000</v>
       </c>
       <c r="P168" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="169" spans="1:16" ht="14.45">
@@ -7144,7 +7195,7 @@
         <v>135</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C169">
         <v>-75.888999999999996</v>
@@ -7156,13 +7207,13 @@
         <v>13.4</v>
       </c>
       <c r="L169" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O169">
         <v>766000</v>
       </c>
       <c r="P169" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="170" spans="1:16" ht="14.45">
@@ -7170,7 +7221,7 @@
         <v>91</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C170">
         <v>-105.08</v>
@@ -7185,7 +7236,7 @@
         <v>17</v>
       </c>
       <c r="P170" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="171" spans="1:16" ht="14.45">
@@ -7193,7 +7244,7 @@
         <v>92</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C171">
         <v>-105.05</v>
@@ -7208,7 +7259,7 @@
         <v>17</v>
       </c>
       <c r="P171" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="172" spans="1:16" ht="14.45">
@@ -7216,7 +7267,7 @@
         <v>93</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C172">
         <v>-105.03</v>
@@ -7231,7 +7282,95 @@
         <v>17</v>
       </c>
       <c r="P172" t="s">
-        <v>209</v>
+        <v>211</v>
+      </c>
+    </row>
+    <row r="173" spans="1:16" ht="15" customHeight="1">
+      <c r="A173">
+        <v>1</v>
+      </c>
+      <c r="B173" t="s">
+        <v>265</v>
+      </c>
+      <c r="C173">
+        <v>-81.86</v>
+      </c>
+      <c r="D173">
+        <v>31.13</v>
+      </c>
+      <c r="E173">
+        <v>15660</v>
+      </c>
+      <c r="F173">
+        <v>12766</v>
+      </c>
+      <c r="G173">
+        <v>54</v>
+      </c>
+      <c r="H173">
+        <v>44</v>
+      </c>
+      <c r="I173">
+        <v>1180</v>
+      </c>
+      <c r="J173">
+        <v>9072</v>
+      </c>
+      <c r="L173" t="s">
+        <v>20</v>
+      </c>
+      <c r="M173" t="s">
+        <v>266</v>
+      </c>
+      <c r="N173">
+        <v>70</v>
+      </c>
+      <c r="P173" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="174" spans="1:16" ht="15" customHeight="1">
+      <c r="A174">
+        <v>2</v>
+      </c>
+      <c r="B174" t="s">
+        <v>268</v>
+      </c>
+      <c r="C174">
+        <v>-82.36</v>
+      </c>
+      <c r="D174">
+        <v>31.28</v>
+      </c>
+      <c r="E174">
+        <v>30489</v>
+      </c>
+      <c r="F174">
+        <v>28327</v>
+      </c>
+      <c r="G174">
+        <v>36</v>
+      </c>
+      <c r="H174">
+        <v>60</v>
+      </c>
+      <c r="I174">
+        <v>738</v>
+      </c>
+      <c r="J174">
+        <v>22144</v>
+      </c>
+      <c r="L174" t="s">
+        <v>20</v>
+      </c>
+      <c r="M174" t="s">
+        <v>266</v>
+      </c>
+      <c r="N174">
+        <v>50</v>
+      </c>
+      <c r="P174" t="s">
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -7247,77 +7386,77 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -7326,8 +7465,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FEA876AF305721488DA47DBFD2ACFB17" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="aedab2b5b7168589e83d55a1a271d795">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="613700a6-52d8-45ba-99cf-babbe92a0eb2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3e3e55907930e16eaf3c0c8f0d4d8a8" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FEA876AF305721488DA47DBFD2ACFB17" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bb2c9507deb23dddadc3a7a145e1d328">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="613700a6-52d8-45ba-99cf-babbe92a0eb2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e2cb7a7579ea1114cd5d791bf8e98040" ns1:_="" ns2:_="">
+    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
     <xsd:import namespace="613700a6-52d8-45ba-99cf-babbe92a0eb2"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -7342,11 +7482,28 @@
                 <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyProperties" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyUIAction" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
         </xsd:sequence>
       </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="_ip_UnifiedCompliancePolicyProperties" ma:index="16" nillable="true" ma:displayName="Unified Compliance Policy Properties" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyProperties">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_ip_UnifiedCompliancePolicyUIAction" ma:index="17" nillable="true" ma:displayName="Unified Compliance Policy UI Action" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyUIAction">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="613700a6-52d8-45ba-99cf-babbe92a0eb2" elementFormDefault="qualified">
@@ -7387,6 +7544,11 @@
     <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="18" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -7502,12 +7664,14 @@
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Notes xmlns="613700a6-52d8-45ba-99cf-babbe92a0eb2" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2275E7B3-2ACA-4DE3-99B0-AD105D2B791B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A634CD8-3C3D-45DC-A2F8-29F07E681EBC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>